<commit_message>
Support 6.23 subframe data layout
</commit_message>
<xml_diff>
--- a/Raw_data/数据格式.xlsx
+++ b/Raw_data/数据格式.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Desktop\AITO_Data_processing_program\Raw_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{798FF65C-2D04-471D-93BE-91EAA23B4EDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{945370A5-40E1-4114-A037-4F485D3F97A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="27">
   <si>
     <t>文件夹命名</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -121,6 +121,18 @@
   </si>
   <si>
     <t>13个（2个三向加速度传感器）：1前排麦克风、2中排麦克风、3后排麦克风、4左半轴x向加速度、5左半轴y向加速度、6左半轴z向加速度、7右半轴x向加速度、8右半轴y向加速度、9右半轴z向加速度、10左前、11左中、12左后、13右前、14右中、15右后、16左动力吸振器、17右动力吸振器</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>6.23</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>副车架试验，无麦克风数据</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>9个：1力传感器、2左输入、3右动力吸振器、4左前、5左中、6左后、7右前、8右中、9右后</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -468,7 +480,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr defaultRowHeight="17.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="16.33203125" style="1" customWidth="1"/>
@@ -612,6 +624,20 @@
         <v>22</v>
       </c>
     </row>
+    <row r="11" spans="1:5" s="3" customFormat="1" ht="62.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="D3:D4"/>

</xml_diff>

<commit_message>
Update 6.23 subframe layout
</commit_message>
<xml_diff>
--- a/Raw_data/数据格式.xlsx
+++ b/Raw_data/数据格式.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Desktop\AITO_Data_processing_program\Raw_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{945370A5-40E1-4114-A037-4F485D3F97A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94627689-A175-427E-9D01-6CEB6FEFC441}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -132,7 +132,7 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>9个：1力传感器、2左输入、3右动力吸振器、4左前、5左中、6左后、7右前、8右中、9右后</t>
+    <t>10个：1力传感器、2右输入、3右动力吸振器、4声子晶体、5左前、6左中、7左后、8右前、9右中、10右后</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -629,7 +629,7 @@
         <v>24</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>26</v>

</xml_diff>